<commit_message>
Add Bible reference + spoiler-free context to Guess the Fake
Each round now shows where it comes from (e.g. "Luke 15") and a one-line
setup that orients players without revealing which statement is fake. Shown
during the guess in both whole-group and teams modes.

- lib/guessTheFake.ts: reference/context on every round (offline fallback)
- v9 migration adds reference/context columns and fills all 85 by topic
- review spreadsheet gains Reference and Context columns

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Guess_the_Fake_Questions.xlsx
+++ b/Guess_the_Fake_Questions.xlsx
@@ -11,7 +11,7 @@
     <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Guess the Fake'!$A$1:$I$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Guess the Fake'!$A$1:$K$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I86"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -518,6 +518,8 @@
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,6 +568,16 @@
           <t>Why it's fake (the truth)</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Context (no spoilers)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -609,6 +621,16 @@
           <t>It rained 40 days and 40 nights, not 100.</t>
         </is>
       </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 6-9</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>God sends a flood but rescues one faithful family.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -652,6 +674,16 @@
           <t>The sun, moon, and stars were made on the fourth day.</t>
         </is>
       </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 1</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>God forms the world and everything in it, step by step.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -695,6 +727,16 @@
           <t>His son Solomon built the temple, not David.</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>1 Samuel 17</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>A shepherd boy steps onto the battlefield against a giant.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -738,6 +780,16 @@
           <t>Jonah ran the opposite way, sailing toward Tarshish.</t>
         </is>
       </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Jonah 1-4</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>God calls a prophet to carry a message to the city of Nineveh.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -781,6 +833,16 @@
           <t>The number of wise men is never given — only three gifts are named.</t>
         </is>
       </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Luke 2; Matthew 2</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>The night Jesus is born and those who come to see him.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -824,6 +886,16 @@
           <t>The fruit is never identified as an apple.</t>
         </is>
       </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 2-3</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>The first people and their choice in the Garden of Eden.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -867,6 +939,16 @@
           <t>That was Joseph. Daniel served kings of Babylon and Persia.</t>
         </is>
       </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Daniel 1; 6</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>A faithful young man stays true to God in a foreign royal court.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -910,6 +992,16 @@
           <t>There were ten commandments.</t>
         </is>
       </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 20</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>God gives his people the laws they are to live by.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -953,6 +1045,16 @@
           <t>His first miracle was turning water into wine at Cana.</t>
         </is>
       </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>John 2; Matthew 14</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>A look at some of the signs and wonders Jesus performed.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -996,6 +1098,16 @@
           <t>He first appeared to Mary Magdalene and the women, not Pilate.</t>
         </is>
       </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 28; John 20</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Easter morning, when the tomb is found empty.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1039,6 +1151,16 @@
           <t>He used the jawbone of a donkey.</t>
         </is>
       </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Judges 13-16</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>A judge of Israel set apart with extraordinary strength.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1082,6 +1204,16 @@
           <t>It was a coat of many colors (a richly ornamented robe).</t>
         </is>
       </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 37-45</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Jacob's favored son, betrayed by his brothers, rises in Egypt.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1125,6 +1257,16 @@
           <t>Moses died first; Joshua led them across the Jordan.</t>
         </is>
       </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 2-3; Deuteronomy 34</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>The leader God chose to free Israel from Egypt.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1168,6 +1310,16 @@
           <t>He came humbly on a donkey, not a war horse.</t>
         </is>
       </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 21</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Jesus arrives in Jerusalem to the cheers of the crowds.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1211,6 +1363,16 @@
           <t>The parable answers the question 'Who is my neighbor?'</t>
         </is>
       </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Luke 10</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>A parable about a traveler left hurt on a dangerous road.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1254,6 +1416,16 @@
           <t>The house on sand collapsed when the storm came.</t>
         </is>
       </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 7</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>A short parable about two builders and where they build.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1297,6 +1469,16 @@
           <t>He searched until he found it, then celebrated.</t>
         </is>
       </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Luke 15</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>A parable about a shepherd missing one of his flock.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1340,6 +1522,16 @@
           <t>That was Zacchaeus, not Peter.</t>
         </is>
       </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 14; 26</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>One of Jesus' twelve disciples and their frequent spokesman.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1383,6 +1575,16 @@
           <t>John was a relative of Jesus, not his twin.</t>
         </is>
       </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 3; Luke 1</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>The prophet who prepared the way for Jesus.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1426,6 +1628,16 @@
           <t>Sarah was about 90 when Isaac was born.</t>
         </is>
       </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 15-22</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>God's promise to make a great nation from one man.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1469,6 +1681,16 @@
           <t>Paul (formerly Saul) was not one of the Twelve; he came later.</t>
         </is>
       </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Acts 9</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>A leading apostle who carried the gospel across the world.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1512,6 +1734,16 @@
           <t>God scattered the people by confusing their language; no fire.</t>
         </is>
       </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 11</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>People unite to build a tower reaching to the heavens.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1555,6 +1787,16 @@
           <t>Esther saved her people through courage before the king, not battle.</t>
         </is>
       </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Esther 4-7</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>A queen faces a deadly plot against her people.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1598,6 +1840,16 @@
           <t>That was his father David.</t>
         </is>
       </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>1 Kings 3-6</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>One of Israel's greatest kings, the son of David.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1641,6 +1893,16 @@
           <t>The plagues included frogs, gnats, flies, and locusts — no spiders.</t>
         </is>
       </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 7-12</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>God sends a series of plagues to free his people.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1684,6 +1946,16 @@
           <t>Judas Iscariot was the betrayer, not Matthew.</t>
         </is>
       </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 10; 26</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>The twelve men Jesus chose to follow him closely.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1727,6 +1999,16 @@
           <t>They wandered for forty years.</t>
         </is>
       </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 16; Numbers 14</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Israel's long journey through the wilderness.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1770,6 +2052,16 @@
           <t>The walls fell after the people shouted and blew trumpets.</t>
         </is>
       </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Joshua 6</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Israel's first battle in the Promised Land.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1813,6 +2105,16 @@
           <t>Ruth was the great-grandmother of King David.</t>
         </is>
       </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Ruth 1-4</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>A loyal widow's story from the days of the judges.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1856,6 +2158,16 @@
           <t>It's reversed: Abel kept flocks and Cain worked the soil.</t>
         </is>
       </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 4</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>The first two brothers and their offerings to God.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1899,6 +2211,16 @@
           <t>He was sold into Egypt and rose to second-in-command.</t>
         </is>
       </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 37</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>The dreams of a young man that stir his brothers' anger.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1942,6 +2264,16 @@
           <t>After his baptism Jesus went into the wilderness to be tempted.</t>
         </is>
       </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 3; Mark 1</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>The day Jesus is baptized as his ministry begins.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1985,6 +2317,16 @@
           <t>Jesus refused to turn stones into bread.</t>
         </is>
       </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 4; Luke 4</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Jesus is tested in the wilderness.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2028,6 +2370,16 @@
           <t>Jesus himself called Lazarus out of the tomb.</t>
         </is>
       </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>John 11</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Two sisters grieve their brother and send for Jesus.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2071,6 +2423,16 @@
           <t>He preached it on a mountainside, which is why it's the Sermon on the Mount.</t>
         </is>
       </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 5-7</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Jesus' most famous block of teaching to his followers.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2114,6 +2476,16 @@
           <t>He gave half to the poor and repaid those he cheated four times over.</t>
         </is>
       </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Luke 19</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>A tax collector climbs to catch a glimpse of Jesus.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2157,6 +2529,16 @@
           <t>His father ran to him and threw a celebration feast.</t>
         </is>
       </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Luke 15</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>A parable about a son who leaves home with his inheritance.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2200,6 +2582,16 @@
           <t>It was 5,000 men, besides women and children.</t>
         </is>
       </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 14; John 6</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>Jesus feeds a huge crowd from a small lunch.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2243,6 +2635,16 @@
           <t>Nicodemus was a Pharisee and ruler of the Jews, not one of the Twelve.</t>
         </is>
       </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>John 3</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>A man comes to Jesus at night with deep questions.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2286,6 +2688,16 @@
           <t>They attacked at night with trumpets, torches, and clay jars.</t>
         </is>
       </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Judges 6-7</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>God calls an unlikely hero to rescue Israel.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2329,6 +2741,16 @@
           <t>God restored Job with double what he had before.</t>
         </is>
       </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Job 1-2; 42</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>A blameless man loses everything and is tested.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2372,6 +2794,16 @@
           <t>Jesus defended Mary's choice to listen to him.</t>
         </is>
       </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Luke 10</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Jesus visits the home of two sisters.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2415,6 +2847,16 @@
           <t>The seed represents the word of God.</t>
         </is>
       </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 13</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>A parable about a farmer scattering seed on different ground.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2458,6 +2900,16 @@
           <t>Judas was the betrayer; Peter would deny knowing Jesus.</t>
         </is>
       </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 26; John 13</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Jesus shares a final meal with his disciples.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2501,6 +2953,16 @@
           <t>He was crucified at Golgotha, 'the place of the skull.'</t>
         </is>
       </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 27; John 19</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>The hours of Jesus' death on the cross.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2544,6 +3006,16 @@
           <t>Jesus appeared and invited Thomas to touch his wounds.</t>
         </is>
       </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>John 20</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>One disciple struggles to believe the others' news.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2587,6 +3059,16 @@
           <t>His name became Paul.</t>
         </is>
       </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Acts 9</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>A fierce enemy of the church meets Jesus on the road.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2630,6 +3112,16 @@
           <t>They walked out unharmed, joined by a mysterious fourth figure.</t>
         </is>
       </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Daniel 3</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Three friends refuse to bow to a king's golden statue.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2673,6 +3165,16 @@
           <t>It was a grave sin that brought judgment, not reward.</t>
         </is>
       </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 32</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>While Moses is on the mountain, the people grow restless.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2716,6 +3218,16 @@
           <t>They came later and found the child in a house, not the stable.</t>
         </is>
       </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 2</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Visitors from the east follow a star to find Jesus.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2759,6 +3271,16 @@
           <t>Jesus asked her for a drink of water.</t>
         </is>
       </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>John 4</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Jesus stops to talk with a woman drawing water.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2802,6 +3324,16 @@
           <t>He went away sad because he had great wealth.</t>
         </is>
       </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Mark 10</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>A wealthy man asks Jesus about eternal life.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2845,6 +3377,16 @@
           <t>Jesus' mother was Mary of Nazareth, a different Mary.</t>
         </is>
       </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>John 20</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>One of the women closest to Jesus during his ministry.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2888,6 +3430,16 @@
           <t>The thankful one was a Samaritan.</t>
         </is>
       </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Luke 17</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Ten sick men cry out to Jesus for healing.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2931,6 +3483,16 @@
           <t>Jesus told him to take up his mat and walk.</t>
         </is>
       </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Mark 2</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Friends go to great lengths to bring a man to Jesus.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2974,6 +3536,16 @@
           <t>Esau was born first; Jacob was the younger twin.</t>
         </is>
       </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 25; 27</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Twin brothers struggle over blessing and birthright.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3017,6 +3589,16 @@
           <t>Isaac had twin sons, Jacob and Esau; Ishmael was Abraham's son.</t>
         </is>
       </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 21-24</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>The long-promised son of Abraham and Sarah.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3060,6 +3642,16 @@
           <t>Aaron was Moses' older brother.</t>
         </is>
       </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 4; 32</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Moses' right-hand man during the exodus.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3103,6 +3695,16 @@
           <t>Adam lived 930 years.</t>
         </is>
       </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 5</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>The long genealogy from Adam through the early generations.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3146,6 +3748,16 @@
           <t>Saul was the first king; David was the second.</t>
         </is>
       </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>1 Samuel 8-10</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>How Israel first came to have kings.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -3189,6 +3801,16 @@
           <t>It was Jonah who was swallowed by the fish.</t>
         </is>
       </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Old Testament prophets</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>A quick tour of several Old Testament prophets.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3232,6 +3854,16 @@
           <t>It was carried by Levites using poles on their shoulders.</t>
         </is>
       </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 25; Numbers 4</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>The sacred golden chest at the center of Israel's worship.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3275,6 +3907,16 @@
           <t>The tribe of Judah descended from Judah, another son of Jacob.</t>
         </is>
       </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 49</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>The sons of Jacob who became the tribes of Israel.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3318,6 +3960,16 @@
           <t>About 3,000 people were added that day.</t>
         </is>
       </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Acts 2</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>The Holy Spirit comes on the believers in Jerusalem.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3361,6 +4013,16 @@
           <t>Stephen was stoned; he was not beheaded.</t>
         </is>
       </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Acts 6-7</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>The first follower of Jesus to die for his faith.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3404,6 +4066,16 @@
           <t>The Spirit carried Philip away to another town — no whale.</t>
         </is>
       </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Acts 8</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Philip meets a foreign official reading Scripture on a road.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3447,6 +4119,16 @@
           <t>It was Jael who killed the enemy commander Sisera with a tent peg.</t>
         </is>
       </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Judges 4-5</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>A prophetess leads Israel in a time of danger.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3490,6 +4172,16 @@
           <t>Moses parted the Red Sea; Joshua later crossed the Jordan River.</t>
         </is>
       </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Joshua 3; 10</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Moses' successor leads Israel into the Promised Land.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3533,6 +4225,16 @@
           <t>They received five, two, and one talent — different amounts.</t>
         </is>
       </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 25</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>A parable about servants entrusted with their master's money.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3576,6 +4278,16 @@
           <t>Moses and Elijah appeared with Jesus, not Abraham and David.</t>
         </is>
       </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 17</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>Jesus is revealed in glory on a mountaintop.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -3619,6 +4331,16 @@
           <t>Judas identified Jesus with a kiss.</t>
         </is>
       </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>Matthew 26</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>Jesus prays in a garden on the night he is arrested.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3662,6 +4384,16 @@
           <t>They recognized him when he broke the bread.</t>
         </is>
       </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>Luke 24</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>Two followers meet a stranger on the road after Easter.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3705,6 +4437,16 @@
           <t>He ascended from the Mount of Olives near Bethany.</t>
         </is>
       </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>Acts 1</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>Jesus' final moments with his disciples before heaven.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3748,6 +4490,16 @@
           <t>A hand wrote on the plaster wall; there's no mention of flames.</t>
         </is>
       </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>Daniel 5</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>A king's banquet is interrupted by a strange sign.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3791,6 +4543,16 @@
           <t>He was the king of Babylon.</t>
         </is>
       </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>Daniel 2; 4</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>A powerful king has troubling dreams and is humbled.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -3834,6 +4596,16 @@
           <t>Rebekah was the mother of the twins Jacob and Esau.</t>
         </is>
       </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 24-25</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>The wife chosen for Isaac at a well.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -3877,6 +4649,16 @@
           <t>He dreamed it in the wilderness, using a stone as a pillow, while fleeing Esau.</t>
         </is>
       </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>Genesis 28</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>Jacob falls asleep and dreams of heaven.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -3920,6 +4702,16 @@
           <t>That was Korah; Miriam was struck with temporary leprosy.</t>
         </is>
       </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>Exodus 15; Numbers 12</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>The sister of Moses and a leader among Israel's women.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3963,6 +4755,16 @@
           <t>Balaam was a diviner hired to curse Israel.</t>
         </is>
       </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>Numbers 22</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>On his journey, this man encounters far more than he expected.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -4006,6 +4808,16 @@
           <t>The walls were finished in just 52 days.</t>
         </is>
       </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>Nehemiah 2-6</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>Rebuilding the broken-down walls of Jerusalem.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -4049,6 +4861,16 @@
           <t>Ezra lived centuries before the Gospels; he didn't write them.</t>
         </is>
       </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>Ezra 7; Nehemiah 8</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>A scribe helps God's people return to his law.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -4092,6 +4914,16 @@
           <t>Simeon was a devout man in the temple, not an innkeeper.</t>
         </is>
       </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>Luke 2</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>Two devout elders who had long awaited the Messiah.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -4135,6 +4967,16 @@
           <t>Jesus healed him and said his faith had made him well.</t>
         </is>
       </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>Mark 10</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>A blind beggar calls out to Jesus by the roadside.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4178,6 +5020,16 @@
           <t>Jesus raised her, saying, 'Little girl, get up.'</t>
         </is>
       </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>Mark 5</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>A desperate father begs Jesus to help his sick child.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -4221,9 +5073,19 @@
           <t>It was youths who mocked Elisha, and bears (not lions) that came out.</t>
         </is>
       </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>2 Kings 2-6</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t>The prophet who took up Elijah's mantle.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I86"/>
+  <autoFilter ref="A1:K86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>